<commit_message>
worked on card art
</commit_message>
<xml_diff>
--- a/Set1Layout.xlsx
+++ b/Set1Layout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spark\Documents\CardGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81ADC286-BDF1-4B27-A361-5B984B084381}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05214B7A-0AF8-4FD6-B08F-9FB2D411445F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
+    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="9960" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="63">
   <si>
     <t>Total Cards</t>
   </si>
@@ -53,27 +53,12 @@
     <t>Off-Site</t>
   </si>
   <si>
-    <t>Titan</t>
-  </si>
-  <si>
     <t>Total</t>
   </si>
   <si>
-    <t>Birds</t>
-  </si>
-  <si>
-    <t>Jester</t>
-  </si>
-  <si>
     <t>Skeleton</t>
   </si>
   <si>
-    <t>Twisted Golem</t>
-  </si>
-  <si>
-    <t>Last Mass</t>
-  </si>
-  <si>
     <t>Morgue</t>
   </si>
   <si>
@@ -95,9 +80,6 @@
     <t>Abyssal Maw</t>
   </si>
   <si>
-    <t>Space</t>
-  </si>
-  <si>
     <t>Greater Crow</t>
   </si>
   <si>
@@ -125,9 +107,6 @@
     <t>Artistic Golem</t>
   </si>
   <si>
-    <t>Specular Robot</t>
-  </si>
-  <si>
     <t>Shifting Golem</t>
   </si>
   <si>
@@ -192,6 +171,60 @@
   </si>
   <si>
     <t>Knife</t>
+  </si>
+  <si>
+    <t>Celestial</t>
+  </si>
+  <si>
+    <t>Randos</t>
+  </si>
+  <si>
+    <t>Specular Golem</t>
+  </si>
+  <si>
+    <t>Reap</t>
+  </si>
+  <si>
+    <t>Jester (2)</t>
+  </si>
+  <si>
+    <t>Twisted Golem (2)</t>
+  </si>
+  <si>
+    <t>Last Mass (3)</t>
+  </si>
+  <si>
+    <t>Grave Digger</t>
+  </si>
+  <si>
+    <t>Pale Mask</t>
+  </si>
+  <si>
+    <t>Melting Idol</t>
+  </si>
+  <si>
+    <t>Cauldron</t>
+  </si>
+  <si>
+    <t>Tomb Crawler (5)</t>
+  </si>
+  <si>
+    <t>Phase Beast (7)</t>
+  </si>
+  <si>
+    <t>Saturn Bear</t>
+  </si>
+  <si>
+    <t>Marked One (10)</t>
+  </si>
+  <si>
+    <t>Wo Venus</t>
+  </si>
+  <si>
+    <t>Mutation</t>
+  </si>
+  <si>
+    <t>Blood Rage</t>
   </si>
 </sst>
 </file>
@@ -613,7 +646,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D28E8B96-7BB2-4669-969C-772D34FF9DED}">
-  <dimension ref="A1:AD9"/>
+  <dimension ref="A1:AC9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.109375" customWidth="1"/>
@@ -622,16 +655,16 @@
     <col min="4" max="4" width="16.88671875" customWidth="1"/>
     <col min="5" max="5" width="18.33203125" customWidth="1"/>
     <col min="6" max="6" width="8.88671875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" customWidth="1"/>
-    <col min="8" max="11" width="15.77734375" customWidth="1"/>
+    <col min="7" max="7" width="9.5546875" customWidth="1"/>
+    <col min="8" max="11" width="17.6640625" customWidth="1"/>
     <col min="12" max="12" width="8.88671875" style="1"/>
-    <col min="13" max="13" width="9.5546875" customWidth="1"/>
-    <col min="14" max="17" width="17.6640625" customWidth="1"/>
+    <col min="14" max="17" width="16.33203125" customWidth="1"/>
     <col min="18" max="18" width="8.88671875" style="1"/>
-    <col min="20" max="23" width="16.33203125" customWidth="1"/>
+    <col min="20" max="23" width="19.44140625" customWidth="1"/>
     <col min="24" max="24" width="8.88671875" style="1"/>
-    <col min="26" max="29" width="19.44140625" customWidth="1"/>
-    <col min="30" max="30" width="8.88671875" style="1"/>
+    <col min="26" max="26" width="14.109375" customWidth="1"/>
+    <col min="27" max="27" width="14" customWidth="1"/>
+    <col min="28" max="28" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:29" x14ac:dyDescent="0.3">
@@ -640,11 +673,11 @@
       </c>
       <c r="B1" s="2">
         <f>SUM(A8,G8,M8,S8,Y8)</f>
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C1" s="8" t="str">
-        <f>"/ 200"</f>
-        <v>/ 200</v>
+        <f>"/ 150"</f>
+        <v>/ 150</v>
       </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.3">
@@ -660,11 +693,9 @@
       <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="s">
-        <v>5</v>
-      </c>
+      <c r="E2" s="4"/>
       <c r="G2" s="6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>2</v>
@@ -675,11 +706,9 @@
       <c r="J2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>5</v>
-      </c>
+      <c r="K2" s="4"/>
       <c r="M2" s="6" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
       <c r="N2" s="4" t="s">
         <v>2</v>
@@ -690,11 +719,9 @@
       <c r="P2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" s="4" t="s">
-        <v>5</v>
-      </c>
+      <c r="Q2" s="4"/>
       <c r="S2" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="T2" s="4" t="s">
         <v>2</v>
@@ -705,11 +732,9 @@
       <c r="V2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="W2" s="4" t="s">
-        <v>5</v>
-      </c>
+      <c r="W2" s="4"/>
       <c r="Y2" s="6" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="Z2" s="4" t="s">
         <v>2</v>
@@ -720,73 +745,59 @@
       <c r="AB2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="AC2" s="4" t="s">
-        <v>5</v>
-      </c>
+      <c r="AC2" s="4"/>
     </row>
     <row r="3" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A3" s="5">
         <f>COUNTA(B3:B60)</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
-        <v>13</v>
-      </c>
       <c r="D3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G3" s="5">
         <f>COUNTA(H3:H60)</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H3" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="I3" t="s">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="J3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K3" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="M3" s="5">
         <f>COUNTA(N3:N60)</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N3" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="O3" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="P3" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="S3" s="5">
         <f>COUNTA(T3:T60)</f>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="T3" t="s">
-        <v>48</v>
+        <v>22</v>
       </c>
       <c r="U3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="V3" t="s">
-        <v>44</v>
-      </c>
-      <c r="W3" t="s">
         <v>35</v>
       </c>
       <c r="Y3" s="5">
@@ -794,204 +805,253 @@
         <v>3</v>
       </c>
       <c r="Z3" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="AA3" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="AB3" t="s">
-        <v>42</v>
-      </c>
-      <c r="AC3" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A4" s="5">
         <f>COUNTA(C3:C60)</f>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>50</v>
+      </c>
+      <c r="C4" t="s">
+        <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="G4" s="5">
         <f>COUNTA(I3:I60)</f>
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H4" t="s">
-        <v>22</v>
+        <v>14</v>
+      </c>
+      <c r="I4" t="s">
+        <v>11</v>
       </c>
       <c r="J4" t="s">
-        <v>26</v>
-      </c>
-      <c r="K4" t="s">
-        <v>45</v>
+        <v>19</v>
       </c>
       <c r="M4" s="5">
         <f>COUNTA(O3:O60)</f>
-        <v>5</v>
+        <v>4</v>
+      </c>
+      <c r="N4" t="s">
+        <v>43</v>
       </c>
       <c r="O4" t="s">
-        <v>16</v>
+        <v>27</v>
+      </c>
+      <c r="P4" t="s">
+        <v>39</v>
       </c>
       <c r="S4" s="5">
         <f>COUNTA(U3:U60)</f>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="T4" t="s">
-        <v>50</v>
-      </c>
-      <c r="U4" t="s">
-        <v>34</v>
-      </c>
-      <c r="V4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="Y4" s="5">
         <f>COUNTA(AA3:AA60)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Z4" t="s">
-        <v>29</v>
-      </c>
-      <c r="AB4" t="s">
-        <v>43</v>
+        <v>6</v>
+      </c>
+      <c r="AA4" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" s="5">
         <f>COUNTA(D3:D60)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>51</v>
+      </c>
+      <c r="C5" t="s">
+        <v>48</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="G5" s="5">
         <f>COUNTA(J3:J60)</f>
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="H5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5" t="s">
+        <v>20</v>
       </c>
       <c r="M5" s="5">
         <f>COUNTA(P3:P60)</f>
-        <v>1</v>
+        <v>3</v>
+      </c>
+      <c r="N5" t="s">
+        <v>28</v>
       </c>
       <c r="O5" t="s">
-        <v>39</v>
+        <v>29</v>
+      </c>
+      <c r="P5" t="s">
+        <v>40</v>
       </c>
       <c r="S5" s="5">
         <f>COUNTA(V3:V60)</f>
-        <v>3</v>
-      </c>
-      <c r="U5" t="s">
-        <v>36</v>
-      </c>
-      <c r="V5" t="s">
-        <v>47</v>
+        <v>1</v>
+      </c>
+      <c r="T5" t="s">
+        <v>23</v>
       </c>
       <c r="Y5" s="5">
         <f>COUNTA(AB3:AB60)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Z5" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A6" s="5">
         <f>COUNTA(E3:E60)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>56</v>
+      </c>
+      <c r="C6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D6" t="s">
+        <v>53</v>
       </c>
       <c r="G6" s="5">
         <f>COUNTA(K3:K60)</f>
-        <v>2</v>
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" t="s">
+        <v>18</v>
       </c>
       <c r="M6" s="5">
         <f>COUNTA(Q3:Q60)</f>
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="N6" t="s">
+        <v>58</v>
       </c>
       <c r="O6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="S6" s="5">
         <f>COUNTA(W3:W60)</f>
-        <v>1</v>
-      </c>
-      <c r="U6" t="s">
-        <v>37</v>
+        <v>0</v>
+      </c>
+      <c r="T6" t="s">
+        <v>24</v>
       </c>
       <c r="Y6" s="5">
         <f>COUNTA(AC3:AC60)</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="B7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D7" t="s">
+        <v>54</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
+      </c>
+      <c r="H7" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" t="s">
+        <v>61</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="O7" t="s">
-        <v>51</v>
+        <v>5</v>
+      </c>
+      <c r="N7" t="s">
+        <v>60</v>
       </c>
       <c r="S7" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="Y7" s="4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A8" s="5">
         <f>SUM(A3:A6)</f>
-        <v>9</v>
+        <v>16</v>
+      </c>
+      <c r="B8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" t="s">
+        <v>55</v>
       </c>
       <c r="G8" s="5">
         <f>SUM(G3:G6)</f>
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="M8" s="5">
         <f>SUM(M3:M6)</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="S8" s="5">
         <f>SUM(S3:S6)</f>
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="Y8" s="5">
         <f>SUM(Y3:Y6)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="G9" s="5">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="M9" s="5">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="S9" s="5">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="Y9" s="5">
-        <v>40</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
made symbols and art
</commit_message>
<xml_diff>
--- a/Set1Layout.xlsx
+++ b/Set1Layout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spark\Documents\CardGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EEAB7BA-18B0-4FB7-995D-70D525FFD598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37D383E-5DD3-4BD3-95EF-457292395262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1884" yWindow="1884" windowWidth="17280" windowHeight="9960" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="73">
   <si>
     <t>Total Cards</t>
   </si>
@@ -164,9 +164,6 @@
     <t>Formal Wizard</t>
   </si>
   <si>
-    <t>Spring Demon</t>
-  </si>
-  <si>
     <t>Clone Element</t>
   </si>
   <si>
@@ -246,6 +243,18 @@
   </si>
   <si>
     <t>Monolith</t>
+  </si>
+  <si>
+    <t>Rock Throw</t>
+  </si>
+  <si>
+    <t>War on Pluto</t>
+  </si>
+  <si>
+    <t>Tranquility</t>
+  </si>
+  <si>
+    <t>Deconstructor</t>
   </si>
 </sst>
 </file>
@@ -694,7 +703,7 @@
       </c>
       <c r="B1" s="2">
         <f>SUM(A8,G8,M8,S8,Y8)</f>
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C1" s="8" t="str">
         <f>"/ 150"</f>
@@ -729,7 +738,7 @@
       </c>
       <c r="K2" s="4"/>
       <c r="M2" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N2" s="4" t="s">
         <v>2</v>
@@ -755,7 +764,7 @@
       </c>
       <c r="W2" s="4"/>
       <c r="Y2" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="Z2" s="4" t="s">
         <v>2</v>
@@ -774,7 +783,7 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" t="s">
         <v>8</v>
@@ -810,7 +819,7 @@
       </c>
       <c r="S3" s="5">
         <f>COUNTA(T3:T60)</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T3" t="s">
         <v>22</v>
@@ -823,10 +832,10 @@
       </c>
       <c r="Y3" s="5">
         <f>COUNTA(Z3:Z60)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z3" t="s">
-        <v>42</v>
+        <v>6</v>
       </c>
       <c r="AA3" t="s">
         <v>32</v>
@@ -841,13 +850,13 @@
         <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G4" s="5">
         <f>COUNTA(I3:I60)</f>
@@ -867,7 +876,7 @@
         <v>4</v>
       </c>
       <c r="N4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="O4" t="s">
         <v>27</v>
@@ -877,23 +886,26 @@
       </c>
       <c r="S4" s="5">
         <f>COUNTA(U3:U60)</f>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T4" t="s">
-        <v>47</v>
+        <v>46</v>
+      </c>
+      <c r="U4" t="s">
+        <v>69</v>
       </c>
       <c r="V4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="Y4" s="5">
         <f>COUNTA(AA3:AA60)</f>
         <v>2</v>
       </c>
       <c r="Z4" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="AA4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.3">
@@ -902,10 +914,10 @@
         <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D5" t="s">
         <v>34</v>
@@ -925,7 +937,7 @@
       </c>
       <c r="M5" s="5">
         <f>COUNTA(P3:P60)</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N5" t="s">
         <v>28</v>
@@ -943,15 +955,15 @@
       <c r="T5" t="s">
         <v>23</v>
       </c>
+      <c r="U5" t="s">
+        <v>71</v>
+      </c>
       <c r="V5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="Y5" s="5">
         <f>COUNTA(AB3:AB60)</f>
         <v>1</v>
-      </c>
-      <c r="Z5" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:29" x14ac:dyDescent="0.3">
@@ -960,13 +972,13 @@
         <v>0</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" t="s">
         <v>52</v>
-      </c>
-      <c r="D6" t="s">
-        <v>53</v>
       </c>
       <c r="G6" s="5">
         <f>COUNTA(K3:K60)</f>
@@ -979,14 +991,14 @@
         <v>18</v>
       </c>
       <c r="J6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="M6" s="5">
         <f>COUNTA(Q3:Q60)</f>
         <v>0</v>
       </c>
       <c r="N6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="O6" t="s">
         <v>30</v>
@@ -1011,10 +1023,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G7" s="4" t="s">
         <v>5</v>
@@ -1023,19 +1035,22 @@
         <v>38</v>
       </c>
       <c r="I7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="M7" s="4" t="s">
         <v>5</v>
       </c>
       <c r="N7" t="s">
-        <v>58</v>
+        <v>57</v>
+      </c>
+      <c r="P7" t="s">
+        <v>70</v>
       </c>
       <c r="S7" s="4" t="s">
         <v>5</v>
       </c>
       <c r="T7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="Y7" s="4" t="s">
         <v>5</v>
@@ -1047,32 +1062,32 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G8" s="5">
         <f>SUM(G3:G6)</f>
         <v>16</v>
       </c>
       <c r="H8" t="s">
+        <v>62</v>
+      </c>
+      <c r="I8" t="s">
         <v>63</v>
-      </c>
-      <c r="I8" t="s">
-        <v>64</v>
       </c>
       <c r="M8" s="5">
         <f>SUM(M3:M6)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="S8" s="5">
         <f>SUM(S3:S6)</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="T8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="Y8" s="5">
         <f>SUM(Y3:Y6)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.3">
@@ -1087,6 +1102,9 @@
       </c>
       <c r="S9" s="5">
         <v>32</v>
+      </c>
+      <c r="T9" t="s">
+        <v>72</v>
       </c>
       <c r="Y9" s="5">
         <v>22</v>

</xml_diff>

<commit_message>
added 4 new cards
</commit_message>
<xml_diff>
--- a/Set1Layout.xlsx
+++ b/Set1Layout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spark\Documents\CardGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E37D383E-5DD3-4BD3-95EF-457292395262}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA6AD4F2-E9D7-44B6-B3F7-F99B411D50FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="75">
   <si>
     <t>Total Cards</t>
   </si>
@@ -255,6 +255,12 @@
   </si>
   <si>
     <t>Deconstructor</t>
+  </si>
+  <si>
+    <t>Big Catch</t>
+  </si>
+  <si>
+    <t>Barier Lord</t>
   </si>
 </sst>
 </file>
@@ -677,40 +683,40 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D28E8B96-7BB2-4669-969C-772D34FF9DED}">
   <dimension ref="A1:AC9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.109375" customWidth="1"/>
-    <col min="2" max="2" width="15.33203125" customWidth="1"/>
-    <col min="3" max="3" width="17.109375" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" customWidth="1"/>
-    <col min="5" max="5" width="18.33203125" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5546875" customWidth="1"/>
-    <col min="8" max="11" width="17.6640625" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" style="1"/>
-    <col min="14" max="17" width="16.33203125" customWidth="1"/>
-    <col min="18" max="18" width="8.88671875" style="1"/>
-    <col min="20" max="23" width="19.44140625" customWidth="1"/>
-    <col min="24" max="24" width="8.88671875" style="1"/>
-    <col min="26" max="26" width="14.109375" customWidth="1"/>
+    <col min="1" max="1" width="11.140625" customWidth="1"/>
+    <col min="2" max="2" width="15.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" customWidth="1"/>
+    <col min="5" max="5" width="18.28515625" customWidth="1"/>
+    <col min="6" max="6" width="8.85546875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" customWidth="1"/>
+    <col min="8" max="11" width="17.7109375" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" style="1"/>
+    <col min="14" max="17" width="16.28515625" customWidth="1"/>
+    <col min="18" max="18" width="8.85546875" style="1"/>
+    <col min="20" max="23" width="19.42578125" customWidth="1"/>
+    <col min="24" max="24" width="8.85546875" style="1"/>
+    <col min="26" max="26" width="14.140625" customWidth="1"/>
     <col min="27" max="27" width="14" customWidth="1"/>
-    <col min="28" max="28" width="13.44140625" customWidth="1"/>
+    <col min="28" max="28" width="13.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2">
         <f>SUM(A8,G8,M8,S8,Y8)</f>
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C1" s="8" t="str">
         <f>"/ 150"</f>
         <v>/ 150</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>1</v>
       </c>
@@ -777,7 +783,7 @@
       </c>
       <c r="AC2" s="4"/>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <f>COUNTA(B3:B60)</f>
         <v>6</v>
@@ -844,7 +850,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <f>COUNTA(C3:C60)</f>
         <v>4</v>
@@ -899,7 +905,7 @@
       </c>
       <c r="Y4" s="5">
         <f>COUNTA(AA3:AA60)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Z4" t="s">
         <v>21</v>
@@ -908,7 +914,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <f>COUNTA(D3:D60)</f>
         <v>5</v>
@@ -950,7 +956,7 @@
       </c>
       <c r="S5" s="5">
         <f>COUNTA(V3:V60)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T5" t="s">
         <v>23</v>
@@ -965,8 +971,11 @@
         <f>COUNTA(AB3:AB60)</f>
         <v>1</v>
       </c>
+      <c r="AA5" t="s">
+        <v>73</v>
+      </c>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6" s="5">
         <f>COUNTA(E3:E60)</f>
         <v>0</v>
@@ -1013,12 +1022,15 @@
       <c r="T6" t="s">
         <v>24</v>
       </c>
+      <c r="V6" t="s">
+        <v>74</v>
+      </c>
       <c r="Y6" s="5">
         <f>COUNTA(AC3:AC60)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
@@ -1056,7 +1068,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
         <f>SUM(A3:A6)</f>
         <v>15</v>
@@ -1080,17 +1092,17 @@
       </c>
       <c r="S8" s="5">
         <f>SUM(S3:S6)</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="T8" t="s">
         <v>65</v>
       </c>
       <c r="Y8" s="5">
         <f>SUM(Y3:Y6)</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:29" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>32</v>
       </c>

</xml_diff>

<commit_message>
moved around crow cards to randos
</commit_message>
<xml_diff>
--- a/Set1Layout.xlsx
+++ b/Set1Layout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spark\Documents\CardGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF4D9AF9-24DB-482C-9CBE-A88820ADCA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C996DA-B52D-4DC3-A8E6-363DCF1FD5E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -194,9 +194,6 @@
     <t>Saturn Bear</t>
   </si>
   <si>
-    <t>Wo Venus</t>
-  </si>
-  <si>
     <t>Mutation</t>
   </si>
   <si>
@@ -303,6 +300,9 @@
   </si>
   <si>
     <t>Cauldron</t>
+  </si>
+  <si>
+    <t>Venus Woman</t>
   </si>
 </sst>
 </file>
@@ -773,43 +773,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D28E8B96-7BB2-4669-969C-772D34FF9DED}">
   <dimension ref="A1:Y11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" style="7" customWidth="1"/>
-    <col min="3" max="3" width="13.85546875" style="7" customWidth="1"/>
-    <col min="4" max="4" width="16.85546875" style="7" customWidth="1"/>
-    <col min="5" max="5" width="2.7109375" style="8" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" style="7" customWidth="1"/>
-    <col min="8" max="8" width="15.5703125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" style="7" customWidth="1"/>
+    <col min="4" max="4" width="16.88671875" style="7" customWidth="1"/>
+    <col min="5" max="5" width="2.6640625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.44140625" style="7" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" style="7" customWidth="1"/>
     <col min="9" max="9" width="16" style="7" customWidth="1"/>
-    <col min="10" max="10" width="2.7109375" style="8" customWidth="1"/>
-    <col min="11" max="11" width="9.85546875" style="1" customWidth="1"/>
-    <col min="12" max="13" width="16.28515625" style="7" customWidth="1"/>
-    <col min="14" max="14" width="13.140625" style="7" customWidth="1"/>
-    <col min="15" max="15" width="2.7109375" style="8" customWidth="1"/>
+    <col min="10" max="10" width="2.6640625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="9.88671875" style="1" customWidth="1"/>
+    <col min="12" max="13" width="16.33203125" style="7" customWidth="1"/>
+    <col min="14" max="14" width="13.109375" style="7" customWidth="1"/>
+    <col min="15" max="15" width="2.6640625" style="8" customWidth="1"/>
     <col min="16" max="16" width="11" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.7109375" style="7" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" style="7" customWidth="1"/>
-    <col min="19" max="19" width="15.5703125" style="7" customWidth="1"/>
-    <col min="20" max="20" width="2.7109375" style="8" customWidth="1"/>
-    <col min="21" max="21" width="10.5703125" style="1" customWidth="1"/>
-    <col min="22" max="22" width="11.85546875" style="7" customWidth="1"/>
+    <col min="17" max="17" width="14.6640625" style="7" customWidth="1"/>
+    <col min="18" max="18" width="16.5546875" style="7" customWidth="1"/>
+    <col min="19" max="19" width="15.5546875" style="7" customWidth="1"/>
+    <col min="20" max="20" width="2.6640625" style="8" customWidth="1"/>
+    <col min="21" max="21" width="10.5546875" style="1" customWidth="1"/>
+    <col min="22" max="22" width="11.88671875" style="7" customWidth="1"/>
     <col min="23" max="23" width="14" style="7" customWidth="1"/>
-    <col min="24" max="24" width="13.42578125" style="7" customWidth="1"/>
+    <col min="24" max="24" width="13.44140625" style="7" customWidth="1"/>
     <col min="25" max="25" width="3" style="8" customWidth="1"/>
-    <col min="26" max="16384" width="9.140625" style="7"/>
+    <col min="26" max="16384" width="9.109375" style="7"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:24" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="str">
         <f>_xlfn.CONCAT("Total: ", SUM(A11,F11,K11,P11,U11))</f>
-        <v>Total: 0</v>
+        <v>Total: 79</v>
       </c>
       <c r="C1" s="12"/>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -871,13 +871,13 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="str">
-        <f>_xlfn.CONCAT("Unit: ", COUNTA(B3:B60))</f>
-        <v>Unit: 6</v>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <f>COUNTA(B3:B60)</f>
+        <v>6</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>7</v>
@@ -885,9 +885,9 @@
       <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="1" t="str">
-        <f>_xlfn.CONCAT("Unit: ", COUNTA(G3:G60))</f>
-        <v>Unit: 7</v>
+      <c r="F3" s="1">
+        <f>COUNTA(G3:G60)</f>
+        <v>3</v>
       </c>
       <c r="G3" s="4" t="s">
         <v>32</v>
@@ -898,9 +898,9 @@
       <c r="I3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="K3" s="1" t="str">
-        <f>_xlfn.CONCAT("Unit: ", COUNTA(L3:L60))</f>
-        <v>Unit: 7</v>
+      <c r="K3" s="1">
+        <f>COUNTA(L3:L60)</f>
+        <v>7</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>40</v>
@@ -911,9 +911,9 @@
       <c r="N3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="P3" s="1" t="str">
-        <f>_xlfn.CONCAT("Unit: ", COUNTA(Q3:Q60))</f>
-        <v>Unit: 9</v>
+      <c r="P3" s="1">
+        <f>COUNTA(Q3:Q60)</f>
+        <v>9</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>21</v>
@@ -922,11 +922,11 @@
         <v>30</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="U3" s="1" t="str">
-        <f>_xlfn.CONCAT("Unit: ", COUNTA(V3:V60))</f>
-        <v>Unit: 1</v>
+        <v>58</v>
+      </c>
+      <c r="U3" s="1">
+        <f>COUNTA(V3:V60)</f>
+        <v>5</v>
       </c>
       <c r="V3" s="2" t="s">
         <v>5</v>
@@ -934,37 +934,40 @@
       <c r="W3" s="4" t="s">
         <v>31</v>
       </c>
+      <c r="X3" s="3" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="str">
-        <f>_xlfn.CONCAT("Spell: ", COUNTA(C3:C60))</f>
-        <v>Spell: 6</v>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <f>COUNTA(C3:C60)</f>
+        <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>42</v>
       </c>
       <c r="D4" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="1">
+        <f>COUNTA(H3:H60)</f>
+        <v>6</v>
+      </c>
+      <c r="G4" s="4" t="s">
         <v>54</v>
-      </c>
-      <c r="F4" s="1" t="str">
-        <f>_xlfn.CONCAT("Spell: ", COUNTA(H3:H60))</f>
-        <v>Spell: 8</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>13</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>10</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="K4" s="1" t="str">
-        <f>_xlfn.CONCAT("Spell: ", COUNTA(M3:M60))</f>
-        <v>Spell: 6</v>
+        <v>19</v>
+      </c>
+      <c r="K4" s="1">
+        <f>COUNTA(M3:M60)</f>
+        <v>6</v>
       </c>
       <c r="L4" s="4" t="s">
         <v>41</v>
@@ -975,34 +978,37 @@
       <c r="N4" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="P4" s="1" t="str">
-        <f>_xlfn.CONCAT("Spell: ", COUNTA(R3:R60))</f>
-        <v>Spell: 4</v>
+      <c r="P4" s="1">
+        <f>COUNTA(R3:R60)</f>
+        <v>4</v>
       </c>
       <c r="Q4" s="4" t="s">
         <v>45</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="U4" s="1" t="str">
-        <f>_xlfn.CONCAT("Spell: ", COUNTA(W3:W60))</f>
-        <v>Spell: 5</v>
+        <v>59</v>
+      </c>
+      <c r="U4" s="1">
+        <f>COUNTA(W3:W60)</f>
+        <v>7</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="W4" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="str">
-        <f>_xlfn.CONCAT("Off-Site: ", COUNTA(D3:D60))</f>
-        <v>Off-Site: 6</v>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <f>COUNTA(D3:D60)</f>
+        <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>46</v>
@@ -1010,22 +1016,19 @@
       <c r="D5" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="1" t="str">
-        <f>_xlfn.CONCAT("Off-Site: ", COUNTA(I3:I60))</f>
-        <v>Off-Site: 3</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>15</v>
+      <c r="F5" s="1">
+        <f>COUNTA(I3:I60)</f>
+        <v>2</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>77</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K5" s="1" t="str">
-        <f>_xlfn.CONCAT("Off-Site: ", COUNTA(N3:N60))</f>
-        <v>Off-Site: 6</v>
+      <c r="K5" s="1">
+        <f>COUNTA(N3:N60)</f>
+        <v>6</v>
       </c>
       <c r="L5" s="4" t="s">
         <v>27</v>
@@ -1036,33 +1039,36 @@
       <c r="N5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="P5" s="1" t="str">
-        <f>_xlfn.CONCAT("Off-Site: ", COUNTA(S3:S60))</f>
-        <v>Off-Site: 5</v>
+      <c r="P5" s="1">
+        <f>COUNTA(S3:S60)</f>
+        <v>5</v>
       </c>
       <c r="Q5" s="2" t="s">
         <v>22</v>
       </c>
       <c r="R5" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="S5" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="U5" s="1" t="str">
-        <f>_xlfn.CONCAT("Off-Site: ", COUNTA(X3:X60))</f>
-        <v>Off-Site: 0</v>
+        <v>65</v>
+      </c>
+      <c r="U5" s="1">
+        <f>COUNTA(X3:X60)</f>
+        <v>1</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>8</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>47</v>
@@ -1071,13 +1077,10 @@
         <v>48</v>
       </c>
       <c r="F6" s="2">
-        <v>7</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>17</v>
+        <v>4</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>51</v>
       </c>
       <c r="K6" s="2">
         <v>5</v>
@@ -1086,10 +1089,10 @@
         <v>50</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P6" s="2">
         <v>8</v>
@@ -1098,24 +1101,27 @@
         <v>23</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="S6" s="2" t="s">
         <v>38</v>
       </c>
       <c r="U6" s="2">
-        <v>2</v>
+        <v>5</v>
+      </c>
+      <c r="V6" s="4" t="s">
+        <v>14</v>
       </c>
       <c r="W6" s="3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>3</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>28</v>
@@ -1124,72 +1130,69 @@
         <v>49</v>
       </c>
       <c r="F7" s="3">
-        <v>6</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K7" s="3">
         <v>6</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="N7" s="4" t="s">
-        <v>80</v>
+        <v>67</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>79</v>
       </c>
       <c r="P7" s="3">
         <v>6</v>
       </c>
       <c r="Q7" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="S7" s="2" t="s">
         <v>35</v>
       </c>
       <c r="U7" s="3">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="V7" s="5" t="s">
+        <v>37</v>
       </c>
       <c r="W7" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A8" s="4">
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="5" t="s">
-        <v>76</v>
-      </c>
       <c r="F8" s="4">
-        <v>4</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>56</v>
+        <v>3</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>57</v>
       </c>
       <c r="K8" s="4">
         <v>6</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>34</v>
@@ -1198,51 +1201,48 @@
         <v>3</v>
       </c>
       <c r="Q8" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="U8" s="4">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A9" s="5">
         <v>3</v>
       </c>
       <c r="F9" s="5">
         <v>1</v>
       </c>
-      <c r="G9" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>79</v>
-      </c>
       <c r="K9" s="5">
         <v>2</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="P9" s="5">
         <v>1</v>
       </c>
       <c r="Q9" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="U9" s="5">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="W9" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A10" s="10" t="s">
         <v>4</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="H10" s="3" t="s">
-        <v>58</v>
-      </c>
       <c r="K10" s="10" t="s">
         <v>4</v>
       </c>
@@ -1250,35 +1250,35 @@
         <v>4</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="U10" s="10" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <f>SUM(A3:A5)</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="F11" s="1">
         <f>SUM(F3:F5)</f>
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K11" s="1">
         <f>SUM(K3:K5)</f>
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="P11" s="1">
         <f>SUM(P3:P5)</f>
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="Q11" s="3" t="s">
         <v>20</v>
       </c>
       <c r="U11" s="1">
         <f>SUM(U3:U5)</f>
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
worked on some formatting for promotional
</commit_message>
<xml_diff>
--- a/Set1Layout.xlsx
+++ b/Set1Layout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spark\Documents\CardGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36F91645-A37F-40E2-B964-8791AE63D7C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F673B60-23EB-42C0-BEA5-04205B342387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="120">
   <si>
     <t>Ghosts</t>
   </si>
@@ -380,28 +380,25 @@
     <t>Spiritual Warlord</t>
   </si>
   <si>
-    <t>40 / Archetype</t>
-  </si>
-  <si>
-    <t>20 Unit</t>
-  </si>
-  <si>
-    <t>12 Spell</t>
-  </si>
-  <si>
-    <t>8 Off-Site</t>
-  </si>
-  <si>
     <t>Common</t>
   </si>
   <si>
-    <t>Rare</t>
-  </si>
-  <si>
-    <t>Epic</t>
-  </si>
-  <si>
     <t>Legend</t>
+  </si>
+  <si>
+    <t>120 C, 48 R, 24 SR, 12 DR = 204</t>
+  </si>
+  <si>
+    <t>48 / Archetype</t>
+  </si>
+  <si>
+    <t>24 Unit</t>
+  </si>
+  <si>
+    <t>14 Spell</t>
+  </si>
+  <si>
+    <t>10 Off-Site</t>
   </si>
 </sst>
 </file>
@@ -438,7 +435,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -493,6 +490,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -521,7 +524,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -547,16 +550,13 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -924,21 +924,24 @@
   <sheetData>
     <row r="1" spans="1:24" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="14" t="str">
-        <f>_xlfn.CONCAT("Total: ", SUM(A11,F11,K11,P11,U11))</f>
-        <v>Total: 144</v>
+        <f>_xlfn.CONCAT("Total: ", SUM(A7,F7,K7,P7,U7))</f>
+        <v>Total: 106</v>
       </c>
       <c r="B1" s="11" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="D1" s="11" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E1" s="17"/>
       <c r="F1" s="11" t="s">
-        <v>116</v>
+        <v>119</v>
+      </c>
+      <c r="H1" s="11" t="s">
+        <v>115</v>
       </c>
       <c r="J1" s="16"/>
       <c r="O1" s="18"/>
@@ -1009,7 +1012,7 @@
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <f>COUNTA(B3:B60)</f>
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>81</v>
@@ -1022,7 +1025,7 @@
       </c>
       <c r="F3" s="1">
         <f>COUNTA(G3:G60)</f>
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G3" s="5" t="s">
         <v>32</v>
@@ -1035,7 +1038,7 @@
       </c>
       <c r="K3" s="1">
         <f>COUNTA(L3:L60)</f>
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>40</v>
@@ -1048,7 +1051,7 @@
       </c>
       <c r="P3" s="1">
         <f>COUNTA(Q3:Q60)</f>
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="Q3" s="2" t="s">
         <v>21</v>
@@ -1076,7 +1079,7 @@
     <row r="4" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <f>COUNTA(C3:C60)</f>
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>82</v>
@@ -1089,7 +1092,7 @@
       </c>
       <c r="F4" s="1">
         <f>COUNTA(H3:H60)</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>54</v>
@@ -1102,7 +1105,7 @@
       </c>
       <c r="K4" s="1">
         <f>COUNTA(M3:M60)</f>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="L4" s="4" t="s">
         <v>41</v>
@@ -1115,7 +1118,7 @@
       </c>
       <c r="P4" s="1">
         <f>COUNTA(R3:R60)</f>
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="Q4" s="4" t="s">
         <v>45</v>
@@ -1143,7 +1146,7 @@
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <f>COUNTA(D3:D60)</f>
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>83</v>
@@ -1156,7 +1159,7 @@
       </c>
       <c r="F5" s="1">
         <f>COUNTA(I3:I60)</f>
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G5" s="5" t="s">
         <v>77</v>
@@ -1169,7 +1172,7 @@
       </c>
       <c r="K5" s="1">
         <f>COUNTA(N3:N60)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="L5" s="5" t="s">
         <v>27</v>
@@ -1178,7 +1181,7 @@
         <v>66</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="P5" s="1">
         <f>COUNTA(S3:S60)</f>
@@ -1208,9 +1211,8 @@
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A6" s="19" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(B3:D28,$E$1), "/", 18)</f>
-        <v>12/18</v>
+      <c r="A6" s="10" t="s">
+        <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>84</v>
@@ -1221,9 +1223,8 @@
       <c r="D6" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="19" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(G3:I28,$E$1), "/", 18)</f>
-        <v>10/18</v>
+      <c r="F6" s="6" t="s">
+        <v>4</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>88</v>
@@ -1234,9 +1235,8 @@
       <c r="I6" s="4" t="s">
         <v>93</v>
       </c>
-      <c r="K6" s="19" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(L3:N28,$E$1), "/", 18)</f>
-        <v>11/18</v>
+      <c r="K6" s="10" t="s">
+        <v>4</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>50</v>
@@ -1247,9 +1247,8 @@
       <c r="N6" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="P6" s="19" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(Q3:S28,$E$1), "/", 18)</f>
-        <v>10/18</v>
+      <c r="P6" s="10" t="s">
+        <v>4</v>
       </c>
       <c r="Q6" s="5" t="s">
         <v>23</v>
@@ -1260,9 +1259,8 @@
       <c r="S6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U6" s="19" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(V3:X28,$E$1), "/", 18)</f>
-        <v>6/18</v>
+      <c r="U6" s="10" t="s">
+        <v>4</v>
       </c>
       <c r="V6" s="4" t="s">
         <v>14</v>
@@ -1275,9 +1273,9 @@
       </c>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A7" s="20" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(B3:D28,$J$1), "/", 10)</f>
-        <v>10/10</v>
+      <c r="A7" s="1">
+        <f>SUM(A3:A5)</f>
+        <v>21</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>85</v>
@@ -1285,12 +1283,12 @@
       <c r="C7" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="20" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(G3:I28,$J$1), "/", 10)</f>
-        <v>8/10</v>
+      <c r="F7" s="1">
+        <f>SUM(F3:F5)</f>
+        <v>21</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>89</v>
@@ -1301,9 +1299,9 @@
       <c r="I7" s="4" t="s">
         <v>98</v>
       </c>
-      <c r="K7" s="20" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(L3:N28,$J$1), "/", 10)</f>
-        <v>7/10</v>
+      <c r="K7" s="1">
+        <f>SUM(K3:K5)</f>
+        <v>22</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>87</v>
@@ -1314,9 +1312,9 @@
       <c r="N7" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="P7" s="20" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(Q3:S28,$J$1), "/", 10)</f>
-        <v>8/10</v>
+      <c r="P7" s="1">
+        <f>SUM(P3:P5)</f>
+        <v>22</v>
       </c>
       <c r="Q7" s="3" t="s">
         <v>56</v>
@@ -1327,9 +1325,9 @@
       <c r="S7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="U7" s="20" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(V3:X28,$J$1), "/", 10)</f>
-        <v>6/10</v>
+      <c r="U7" s="1">
+        <f>SUM(U3:U5)</f>
+        <v>20</v>
       </c>
       <c r="V7" s="5" t="s">
         <v>37</v>
@@ -1342,10 +1340,7 @@
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(B3:D28,$O$1), "/", 7)</f>
-        <v>7/7</v>
-      </c>
+      <c r="A8" s="22"/>
       <c r="B8" s="5" t="s">
         <v>86</v>
       </c>
@@ -1355,49 +1350,32 @@
       <c r="D8" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="F8" s="21" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(G3:I28,$O$1), "/", 7)</f>
-        <v>7/7</v>
-      </c>
+      <c r="F8" s="22"/>
       <c r="G8" s="2" t="s">
         <v>91</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="K8" s="21" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(L3:N28,$O$1), "/", 7)</f>
-        <v>7/7</v>
-      </c>
+      <c r="I8" s="20"/>
+      <c r="K8" s="22"/>
       <c r="L8" s="3" t="s">
         <v>68</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="P8" s="21" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(Q3:S28,$O$1), "/", 7)</f>
-        <v>7/7</v>
-      </c>
+      <c r="P8" s="22"/>
       <c r="Q8" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="R8" s="4" t="s">
-        <v>119</v>
-      </c>
+      <c r="R8" s="19"/>
       <c r="S8" s="3" t="s">
         <v>105</v>
       </c>
-      <c r="U8" s="21" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(V3:X28,$O$1), "/", 7)</f>
-        <v>4/7</v>
-      </c>
       <c r="V8" s="2" t="s">
         <v>106</v>
       </c>
@@ -1406,59 +1384,34 @@
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" s="5" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(B3:D28,$T$1), "/", 5)</f>
-        <v>5/5</v>
-      </c>
+      <c r="A9" s="23"/>
       <c r="B9" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="F9" s="5" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(G3:I28,$T$1), "/", 5)</f>
-        <v>5/5</v>
-      </c>
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="F9" s="23"/>
       <c r="G9" s="4" t="s">
         <v>92</v>
       </c>
       <c r="H9" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="I9" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="K9" s="5" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(L3:N28,$T$1), "/", 5)</f>
-        <v>5/5</v>
-      </c>
+      <c r="I9" s="19"/>
+      <c r="K9" s="23"/>
       <c r="L9" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="M9" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="M9" s="19"/>
       <c r="N9" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="P9" s="5" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(Q3:S28,$T$1), "/", 5)</f>
-        <v>5/5</v>
-      </c>
+      <c r="P9" s="23"/>
       <c r="Q9" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="R9" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="U9" s="5" t="str">
-        <f>_xlfn.CONCAT(COUNT_COLOR(V3:X28,$T$1), "/", 5)</f>
-        <v>4/5</v>
-      </c>
+      <c r="R9" s="19"/>
+      <c r="U9" s="23"/>
       <c r="V9" s="5" t="s">
         <v>109</v>
       </c>
@@ -1467,181 +1420,89 @@
       </c>
     </row>
     <row r="10" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A10" s="10" t="s">
-        <v>4</v>
-      </c>
+      <c r="A10" s="21"/>
       <c r="B10" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>4</v>
-      </c>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="F10" s="21"/>
       <c r="G10" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="H10" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="I10" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="K10" s="10" t="s">
-        <v>4</v>
-      </c>
+      <c r="H10" s="20"/>
+      <c r="I10" s="19"/>
+      <c r="K10" s="21"/>
       <c r="L10" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="M10" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="M10" s="19"/>
       <c r="N10" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="P10" s="10" t="s">
-        <v>4</v>
-      </c>
+      <c r="P10" s="21"/>
       <c r="Q10" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="R10" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="U10" s="10" t="s">
-        <v>4</v>
-      </c>
+      <c r="R10" s="19"/>
+      <c r="U10" s="21"/>
       <c r="W10" s="3" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="11" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A11" s="1">
-        <f>SUM(A3:A5)</f>
-        <v>34</v>
-      </c>
       <c r="B11" s="4" t="s">
         <v>112</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="F11" s="1">
-        <f>SUM(F3:F5)</f>
-        <v>30</v>
-      </c>
+      <c r="C11" s="19"/>
+      <c r="D11" s="19"/>
       <c r="G11" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="H11" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="K11" s="1">
-        <f>SUM(K3:K5)</f>
-        <v>30</v>
-      </c>
-      <c r="L11" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="M11" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="N11" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="P11" s="1">
-        <f>SUM(P3:P5)</f>
-        <v>30</v>
-      </c>
+      <c r="H11" s="19"/>
+      <c r="L11" s="19"/>
+      <c r="M11" s="19"/>
+      <c r="N11" s="19"/>
       <c r="Q11" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="R11" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="U11" s="1">
-        <f>SUM(U3:U5)</f>
-        <v>20</v>
-      </c>
+      <c r="R11" s="20"/>
     </row>
     <row r="12" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B12" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="L12" s="4" t="s">
-        <v>119</v>
-      </c>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="20"/>
+      <c r="G12" s="19"/>
+      <c r="L12" s="19"/>
       <c r="Q12" s="2" t="s">
         <v>97</v>
       </c>
     </row>
     <row r="13" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B13" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="L13" s="5" t="s">
-        <v>120</v>
-      </c>
+      <c r="B13" s="19"/>
+      <c r="C13" s="20"/>
+      <c r="G13" s="19"/>
+      <c r="L13" s="20"/>
       <c r="Q13" s="2" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B14" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="Q14" s="4" t="s">
-        <v>119</v>
-      </c>
+      <c r="B14" s="20"/>
+      <c r="G14" s="19"/>
+      <c r="L14" s="19"/>
+      <c r="Q14" s="19"/>
     </row>
     <row r="15" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B15" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="Q15" s="4" t="s">
-        <v>119</v>
-      </c>
+      <c r="B15" s="19"/>
+      <c r="G15" s="19"/>
+      <c r="Q15" s="19"/>
     </row>
     <row r="16" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="Q16" s="2" t="s">
-        <v>117</v>
-      </c>
+      <c r="Q16" s="19"/>
     </row>
     <row r="17" spans="17:17" x14ac:dyDescent="0.3">
-      <c r="Q17" s="5" t="s">
-        <v>120</v>
-      </c>
+      <c r="Q17" s="20"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
unified docs into 1
</commit_message>
<xml_diff>
--- a/Set1Layout.xlsx
+++ b/Set1Layout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spark\Documents\CardGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F673B60-23EB-42C0-BEA5-04205B342387}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1BB75D7-8864-48E9-B67B-CADA2AFC5618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="131">
   <si>
     <t>Ghosts</t>
   </si>
@@ -380,32 +380,65 @@
     <t>Spiritual Warlord</t>
   </si>
   <si>
-    <t>Common</t>
-  </si>
-  <si>
-    <t>Legend</t>
-  </si>
-  <si>
-    <t>120 C, 48 R, 24 SR, 12 DR = 204</t>
-  </si>
-  <si>
-    <t>48 / Archetype</t>
-  </si>
-  <si>
-    <t>24 Unit</t>
-  </si>
-  <si>
-    <t>14 Spell</t>
-  </si>
-  <si>
-    <t>10 Off-Site</t>
+    <t>Flesh Ritual</t>
+  </si>
+  <si>
+    <t>Withering Shrine</t>
+  </si>
+  <si>
+    <t>36 / Archetype, 19 C, 9 R, 5 SR, 3 DR</t>
+  </si>
+  <si>
+    <t>Fungal Guardian</t>
+  </si>
+  <si>
+    <t>Apple Guard</t>
+  </si>
+  <si>
+    <t>Ring Generator</t>
+  </si>
+  <si>
+    <t>Madness Policy</t>
+  </si>
+  <si>
+    <t>Last Chance</t>
+  </si>
+  <si>
+    <t>Marlita Blue</t>
+  </si>
+  <si>
+    <t>Marlita Grey</t>
+  </si>
+  <si>
+    <t>Marlita White</t>
+  </si>
+  <si>
+    <t>Marlita Black</t>
+  </si>
+  <si>
+    <t>Marlita Red</t>
+  </si>
+  <si>
+    <t>Marlita Yellow</t>
+  </si>
+  <si>
+    <t>Marlita R-B</t>
+  </si>
+  <si>
+    <t>Come Marlita</t>
+  </si>
+  <si>
+    <t>Marlita Home</t>
+  </si>
+  <si>
+    <t>Marlita Shrine</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -424,12 +457,6 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -524,39 +551,42 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -896,613 +926,697 @@
   <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" style="7" customWidth="1"/>
-    <col min="3" max="3" width="13.88671875" style="7" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" style="7" customWidth="1"/>
-    <col min="5" max="5" width="2.6640625" style="8" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="13.88671875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="16.88671875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="2.6640625" style="6" customWidth="1"/>
     <col min="6" max="6" width="10.44140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" style="7" customWidth="1"/>
-    <col min="8" max="8" width="15.5546875" style="7" customWidth="1"/>
-    <col min="9" max="9" width="16" style="7" customWidth="1"/>
-    <col min="10" max="10" width="2.6640625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="15.44140625" style="5" customWidth="1"/>
+    <col min="8" max="8" width="15.5546875" style="5" customWidth="1"/>
+    <col min="9" max="9" width="16" style="5" customWidth="1"/>
+    <col min="10" max="10" width="2.6640625" style="6" customWidth="1"/>
     <col min="11" max="11" width="9.88671875" style="1" customWidth="1"/>
-    <col min="12" max="13" width="16.33203125" style="7" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" style="7" customWidth="1"/>
-    <col min="15" max="15" width="2.6640625" style="8" customWidth="1"/>
+    <col min="12" max="13" width="16.33203125" style="5" customWidth="1"/>
+    <col min="14" max="14" width="13.109375" style="5" customWidth="1"/>
+    <col min="15" max="15" width="2.6640625" style="6" customWidth="1"/>
     <col min="16" max="16" width="11" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.6640625" style="7" customWidth="1"/>
-    <col min="18" max="18" width="16.5546875" style="7" customWidth="1"/>
-    <col min="19" max="19" width="15.5546875" style="7" customWidth="1"/>
-    <col min="20" max="20" width="2.6640625" style="8" customWidth="1"/>
+    <col min="17" max="17" width="14.6640625" style="5" customWidth="1"/>
+    <col min="18" max="18" width="16.5546875" style="5" customWidth="1"/>
+    <col min="19" max="19" width="15.5546875" style="5" customWidth="1"/>
+    <col min="20" max="20" width="2.6640625" style="6" customWidth="1"/>
     <col min="21" max="21" width="10.5546875" style="1" customWidth="1"/>
-    <col min="22" max="22" width="11.88671875" style="7" customWidth="1"/>
-    <col min="23" max="23" width="14" style="7" customWidth="1"/>
-    <col min="24" max="24" width="13.44140625" style="7" customWidth="1"/>
-    <col min="25" max="25" width="3" style="8" customWidth="1"/>
-    <col min="26" max="16384" width="9.109375" style="7"/>
+    <col min="22" max="22" width="11.88671875" style="5" customWidth="1"/>
+    <col min="23" max="23" width="14" style="5" customWidth="1"/>
+    <col min="24" max="24" width="13.44140625" style="5" customWidth="1"/>
+    <col min="25" max="25" width="3" style="6" customWidth="1"/>
+    <col min="26" max="16384" width="9.109375" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="11" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="14" t="str">
+    <row r="1" spans="1:25" s="8" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="10" t="str">
         <f>_xlfn.CONCAT("Total: ", SUM(A7,F7,K7,P7,U7))</f>
-        <v>Total: 106</v>
-      </c>
-      <c r="B1" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="E1" s="17"/>
-      <c r="F1" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="H1" s="11" t="s">
+        <v>Total: 121</v>
+      </c>
+      <c r="B1" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="J1" s="16"/>
-      <c r="O1" s="18"/>
-      <c r="T1" s="5"/>
+      <c r="C1" s="9"/>
+      <c r="E1" s="12"/>
+      <c r="J1" s="11"/>
+      <c r="O1" s="13"/>
+      <c r="T1" s="4"/>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="C2" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="E2" s="19"/>
+      <c r="F2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="10" t="s">
+      <c r="H2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="K2" s="9" t="s">
+      <c r="J2" s="19"/>
+      <c r="K2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="L2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="M2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="P2" s="9" t="s">
+      <c r="O2" s="19"/>
+      <c r="P2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="10" t="s">
+      <c r="Q2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="10" t="s">
+      <c r="R2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="S2" s="10" t="s">
+      <c r="S2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="U2" s="9" t="s">
+      <c r="T2" s="19"/>
+      <c r="U2" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="V2" s="10" t="s">
+      <c r="V2" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="W2" s="10" t="s">
+      <c r="W2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="X2" s="10" t="s">
+      <c r="X2" s="17" t="s">
         <v>3</v>
       </c>
+      <c r="Y2" s="19"/>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
+    <row r="3" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="15">
         <f>COUNTA(B3:B60)</f>
         <v>9</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="21" t="s">
         <v>81</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="1">
+      <c r="E3" s="19"/>
+      <c r="F3" s="15">
         <f>COUNTA(G3:G60)</f>
+        <v>10</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="J3" s="19"/>
+      <c r="K3" s="15">
+        <f>COUNTA(L3:L60)</f>
         <v>9</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="K3" s="1">
-        <f>COUNTA(L3:L60)</f>
-        <v>8</v>
-      </c>
-      <c r="L3" s="2" t="s">
+      <c r="L3" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="M3" s="4" t="s">
+      <c r="M3" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="21" t="s">
         <v>36</v>
       </c>
-      <c r="P3" s="1">
+      <c r="O3" s="19"/>
+      <c r="P3" s="15">
         <f>COUNTA(Q3:Q60)</f>
         <v>11</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R3" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="S3" s="4" t="s">
+      <c r="S3" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="U3" s="1">
+      <c r="T3" s="19"/>
+      <c r="U3" s="15">
         <f>COUNTA(V3:V60)</f>
+        <v>14</v>
+      </c>
+      <c r="V3" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="W3" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="X3" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="Y3" s="19"/>
+    </row>
+    <row r="4" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="15">
+        <f>COUNTA(C3:C60)</f>
         <v>7</v>
       </c>
-      <c r="V3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="W3" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="X3" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <f>COUNTA(C3:C60)</f>
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="1">
+      <c r="E4" s="19"/>
+      <c r="F4" s="15">
         <f>COUNTA(H3:H60)</f>
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="H4" s="4" t="s">
+      <c r="H4" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="K4" s="1">
+      <c r="J4" s="19"/>
+      <c r="K4" s="15">
         <f>COUNTA(M3:M60)</f>
-        <v>6</v>
-      </c>
-      <c r="L4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="L4" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="N4" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="P4" s="1">
+      <c r="O4" s="19"/>
+      <c r="P4" s="15">
         <f>COUNTA(R3:R60)</f>
         <v>5</v>
       </c>
-      <c r="Q4" s="4" t="s">
+      <c r="Q4" s="22" t="s">
         <v>45</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="R4" s="21" t="s">
         <v>60</v>
       </c>
-      <c r="S4" s="4" t="s">
+      <c r="S4" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="U4" s="1">
+      <c r="T4" s="19"/>
+      <c r="U4" s="15">
         <f>COUNTA(W3:W60)</f>
-        <v>8</v>
-      </c>
-      <c r="V4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="V4" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="W4" s="2" t="s">
+      <c r="W4" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="X4" s="4" t="s">
+      <c r="X4" s="22" t="s">
         <v>107</v>
       </c>
+      <c r="Y4" s="19"/>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5" s="1">
+    <row r="5" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="15">
         <f>COUNTA(D3:D60)</f>
-        <v>6</v>
-      </c>
-      <c r="B5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="22" t="s">
         <v>83</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="1">
+      <c r="E5" s="19"/>
+      <c r="F5" s="15">
         <f>COUNTA(I3:I60)</f>
         <v>5</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="25" t="s">
         <v>77</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="I5" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="K5" s="1">
+      <c r="J5" s="19"/>
+      <c r="K5" s="15">
         <f>COUNTA(N3:N60)</f>
         <v>8</v>
       </c>
-      <c r="L5" s="5" t="s">
+      <c r="L5" s="25" t="s">
         <v>27</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="M5" s="21" t="s">
         <v>66</v>
       </c>
-      <c r="N5" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="P5" s="1">
+      <c r="N5" s="21" t="s">
+        <v>118</v>
+      </c>
+      <c r="O5" s="19"/>
+      <c r="P5" s="15">
         <f>COUNTA(S3:S60)</f>
         <v>6</v>
       </c>
-      <c r="Q5" s="2" t="s">
+      <c r="Q5" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="R5" s="3" t="s">
+      <c r="R5" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="S5" s="5" t="s">
+      <c r="S5" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="U5" s="1">
+      <c r="T5" s="19"/>
+      <c r="U5" s="15">
         <f>COUNTA(X3:X60)</f>
-        <v>5</v>
-      </c>
-      <c r="V5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="V5" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="W5" s="3" t="s">
+      <c r="W5" s="16" t="s">
         <v>64</v>
       </c>
-      <c r="X5" s="5" t="s">
+      <c r="X5" s="25" t="s">
         <v>108</v>
       </c>
+      <c r="Y5" s="19"/>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+    <row r="6" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="E6" s="19"/>
+      <c r="F6" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="I6" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="K6" s="10" t="s">
+      <c r="J6" s="19"/>
+      <c r="K6" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="L6" s="2" t="s">
+      <c r="L6" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="M6" s="2" t="s">
+      <c r="M6" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="N6" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="P6" s="10" t="s">
+      <c r="O6" s="19"/>
+      <c r="P6" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="Q6" s="5" t="s">
+      <c r="Q6" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="R6" s="4" t="s">
+      <c r="R6" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="S6" s="2" t="s">
+      <c r="S6" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="U6" s="10" t="s">
+      <c r="T6" s="19"/>
+      <c r="U6" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="V6" s="4" t="s">
+      <c r="V6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="W6" s="3" t="s">
+      <c r="W6" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="X6" s="5" t="s">
+      <c r="X6" s="25" t="s">
         <v>110</v>
       </c>
+      <c r="Y6" s="19"/>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A7" s="1">
+    <row r="7" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="15">
         <f>SUM(A3:A5)</f>
-        <v>21</v>
-      </c>
-      <c r="B7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" s="16" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="22" t="s">
         <v>49</v>
       </c>
-      <c r="F7" s="1">
+      <c r="E7" s="19"/>
+      <c r="F7" s="15">
         <f>SUM(F3:F5)</f>
-        <v>21</v>
-      </c>
-      <c r="G7" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H7" s="21" t="s">
         <v>55</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="K7" s="1">
+      <c r="J7" s="19"/>
+      <c r="K7" s="15">
         <f>SUM(K3:K5)</f>
         <v>22</v>
       </c>
-      <c r="L7" s="2" t="s">
+      <c r="L7" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="M7" s="4" t="s">
+      <c r="M7" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="N7" s="5" t="s">
+      <c r="N7" s="25" t="s">
         <v>79</v>
       </c>
-      <c r="P7" s="1">
+      <c r="O7" s="19"/>
+      <c r="P7" s="15">
         <f>SUM(P3:P5)</f>
         <v>22</v>
       </c>
-      <c r="Q7" s="3" t="s">
+      <c r="Q7" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="R7" s="5" t="s">
+      <c r="R7" s="25" t="s">
         <v>102</v>
       </c>
-      <c r="S7" s="2" t="s">
+      <c r="S7" s="21" t="s">
         <v>35</v>
       </c>
-      <c r="U7" s="1">
+      <c r="T7" s="19"/>
+      <c r="U7" s="15">
         <f>SUM(U3:U5)</f>
+        <v>32</v>
+      </c>
+      <c r="V7" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="W7" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="X7" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="Y7" s="19"/>
+    </row>
+    <row r="8" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="24"/>
+      <c r="B8" s="25" t="s">
+        <v>86</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="19"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="H8" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="J8" s="19"/>
+      <c r="K8" s="24"/>
+      <c r="L8" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="M8" s="26"/>
+      <c r="N8" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="O8" s="19"/>
+      <c r="P8" s="24"/>
+      <c r="Q8" s="16" t="s">
+        <v>80</v>
+      </c>
+      <c r="S8" s="16" t="s">
+        <v>105</v>
+      </c>
+      <c r="T8" s="19"/>
+      <c r="U8" s="15"/>
+      <c r="V8" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="W8" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="X8" s="21" t="s">
+        <v>129</v>
+      </c>
+      <c r="Y8" s="19"/>
+    </row>
+    <row r="9" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="25"/>
+      <c r="B9" s="21" t="s">
+        <v>100</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="E9" s="19"/>
+      <c r="F9" s="25"/>
+      <c r="G9" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" s="16" t="s">
+        <v>94</v>
+      </c>
+      <c r="J9" s="19"/>
+      <c r="K9" s="25"/>
+      <c r="L9" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="N9" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="O9" s="19"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="T9" s="19"/>
+      <c r="U9" s="25"/>
+      <c r="V9" s="25" t="s">
+        <v>109</v>
+      </c>
+      <c r="W9" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="X9" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="Y9" s="19"/>
+    </row>
+    <row r="10" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="25"/>
+      <c r="B10" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="E10" s="19"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="21" t="s">
+        <v>95</v>
+      </c>
+      <c r="J10" s="19"/>
+      <c r="K10" s="25"/>
+      <c r="L10" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="N10" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="O10" s="19"/>
+      <c r="P10" s="25"/>
+      <c r="Q10" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="T10" s="19"/>
+      <c r="U10" s="25"/>
+      <c r="V10" s="21" t="s">
+        <v>122</v>
+      </c>
+      <c r="W10" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="Y10" s="19"/>
+    </row>
+    <row r="11" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="15"/>
+      <c r="B11" s="25" t="s">
+        <v>112</v>
+      </c>
+      <c r="E11" s="19"/>
+      <c r="F11" s="15"/>
+      <c r="G11" s="21" t="s">
+        <v>96</v>
+      </c>
+      <c r="J11" s="19"/>
+      <c r="K11" s="15"/>
+      <c r="L11" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="O11" s="19"/>
+      <c r="P11" s="15"/>
+      <c r="Q11" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="V7" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="W7" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="X7" s="3" t="s">
-        <v>12</v>
-      </c>
+      <c r="T11" s="19"/>
+      <c r="U11" s="15"/>
+      <c r="V11" s="21" t="s">
+        <v>121</v>
+      </c>
+      <c r="W11" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="Y11" s="19"/>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A8" s="22"/>
-      <c r="B8" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="F8" s="22"/>
-      <c r="G8" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="I8" s="20"/>
-      <c r="K8" s="22"/>
-      <c r="L8" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="M8" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="N8" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="P8" s="22"/>
-      <c r="Q8" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="R8" s="19"/>
-      <c r="S8" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="V8" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="W8" s="2" t="s">
-        <v>78</v>
-      </c>
+    <row r="12" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="15"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="15"/>
+      <c r="G12" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="J12" s="19"/>
+      <c r="K12" s="15"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="15"/>
+      <c r="Q12" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="T12" s="19"/>
+      <c r="U12" s="15"/>
+      <c r="V12" s="21" t="s">
+        <v>123</v>
+      </c>
+      <c r="W12" s="16" t="s">
+        <v>120</v>
+      </c>
+      <c r="Y12" s="19"/>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" s="23"/>
-      <c r="B9" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="C9" s="19"/>
-      <c r="D9" s="19"/>
-      <c r="F9" s="23"/>
-      <c r="G9" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="I9" s="19"/>
-      <c r="K9" s="23"/>
-      <c r="L9" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="M9" s="19"/>
-      <c r="N9" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="P9" s="23"/>
-      <c r="Q9" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="R9" s="19"/>
-      <c r="U9" s="23"/>
-      <c r="V9" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="W9" s="3" t="s">
-        <v>17</v>
-      </c>
+    <row r="13" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="15"/>
+      <c r="E13" s="19"/>
+      <c r="F13" s="15"/>
+      <c r="J13" s="19"/>
+      <c r="K13" s="15"/>
+      <c r="O13" s="19"/>
+      <c r="P13" s="15"/>
+      <c r="Q13" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="T13" s="19"/>
+      <c r="U13" s="15"/>
+      <c r="V13" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="W13" s="16" t="s">
+        <v>128</v>
+      </c>
+      <c r="Y13" s="19"/>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A10" s="21"/>
-      <c r="B10" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="C10" s="19"/>
-      <c r="D10" s="19"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="H10" s="20"/>
-      <c r="I10" s="19"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="M10" s="19"/>
-      <c r="N10" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="P10" s="21"/>
-      <c r="Q10" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="R10" s="19"/>
-      <c r="U10" s="21"/>
-      <c r="W10" s="3" t="s">
-        <v>111</v>
-      </c>
+    <row r="14" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="15"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="15"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="15"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="15"/>
+      <c r="T14" s="19"/>
+      <c r="U14" s="15"/>
+      <c r="V14" s="21" t="s">
+        <v>125</v>
+      </c>
+      <c r="Y14" s="19"/>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B11" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="G11" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="H11" s="19"/>
-      <c r="L11" s="19"/>
-      <c r="M11" s="19"/>
-      <c r="N11" s="19"/>
-      <c r="Q11" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="R11" s="20"/>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="V15" s="2" t="s">
+        <v>126</v>
+      </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="20"/>
-      <c r="G12" s="19"/>
-      <c r="L12" s="19"/>
-      <c r="Q12" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B13" s="19"/>
-      <c r="C13" s="20"/>
-      <c r="G13" s="19"/>
-      <c r="L13" s="20"/>
-      <c r="Q13" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B14" s="20"/>
-      <c r="G14" s="19"/>
-      <c r="L14" s="19"/>
-      <c r="Q14" s="19"/>
-    </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="B15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="Q15" s="19"/>
-    </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="Q16" s="19"/>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="V16" s="3" t="s">
+        <v>127</v>
+      </c>
     </row>
     <row r="17" spans="17:17" x14ac:dyDescent="0.3">
-      <c r="Q17" s="20"/>
+      <c r="Q17" s="14"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
implemented the draft tool properly, added cards up to plague
</commit_message>
<xml_diff>
--- a/Set1Layout.xlsx
+++ b/Set1Layout.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spark\Documents\CardGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1BB75D7-8864-48E9-B67B-CADA2AFC5618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2154F625-4C11-4059-8CDF-EA7FD261F6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15345" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -551,7 +551,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -571,27 +571,94 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="9">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFCAEDFB"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE49EDD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFE49EDD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF7C7AC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF7C7AC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF7C7AC"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDAF2D0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDAF2D0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDAF2D0"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -923,36 +990,36 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D28E8B96-7BB2-4669-969C-772D34FF9DED}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Y17"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="1" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="13.88671875" style="5" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" style="5" customWidth="1"/>
-    <col min="5" max="5" width="2.6640625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="10.44140625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="15.44140625" style="5" customWidth="1"/>
-    <col min="8" max="8" width="15.5546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="14.42578125" style="5" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" style="5" customWidth="1"/>
+    <col min="4" max="4" width="16.85546875" style="5" customWidth="1"/>
+    <col min="5" max="5" width="2.7109375" style="6" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" style="5" customWidth="1"/>
+    <col min="8" max="8" width="15.5703125" style="5" customWidth="1"/>
     <col min="9" max="9" width="16" style="5" customWidth="1"/>
-    <col min="10" max="10" width="2.6640625" style="6" customWidth="1"/>
-    <col min="11" max="11" width="9.88671875" style="1" customWidth="1"/>
-    <col min="12" max="13" width="16.33203125" style="5" customWidth="1"/>
-    <col min="14" max="14" width="13.109375" style="5" customWidth="1"/>
-    <col min="15" max="15" width="2.6640625" style="6" customWidth="1"/>
+    <col min="10" max="10" width="2.7109375" style="6" customWidth="1"/>
+    <col min="11" max="11" width="9.85546875" style="1" customWidth="1"/>
+    <col min="12" max="13" width="16.28515625" style="5" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" style="5" customWidth="1"/>
+    <col min="15" max="15" width="2.7109375" style="6" customWidth="1"/>
     <col min="16" max="16" width="11" style="1" customWidth="1"/>
-    <col min="17" max="17" width="14.6640625" style="5" customWidth="1"/>
-    <col min="18" max="18" width="16.5546875" style="5" customWidth="1"/>
-    <col min="19" max="19" width="15.5546875" style="5" customWidth="1"/>
-    <col min="20" max="20" width="2.6640625" style="6" customWidth="1"/>
-    <col min="21" max="21" width="10.5546875" style="1" customWidth="1"/>
-    <col min="22" max="22" width="11.88671875" style="5" customWidth="1"/>
+    <col min="17" max="17" width="14.7109375" style="5" customWidth="1"/>
+    <col min="18" max="18" width="16.5703125" style="5" customWidth="1"/>
+    <col min="19" max="19" width="15.5703125" style="5" customWidth="1"/>
+    <col min="20" max="20" width="2.7109375" style="6" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" style="1" customWidth="1"/>
+    <col min="22" max="22" width="11.85546875" style="5" customWidth="1"/>
     <col min="23" max="23" width="14" style="5" customWidth="1"/>
-    <col min="24" max="24" width="13.44140625" style="5" customWidth="1"/>
+    <col min="24" max="24" width="13.42578125" style="5" customWidth="1"/>
     <col min="25" max="25" width="3" style="6" customWidth="1"/>
-    <col min="26" max="16384" width="9.109375" style="5"/>
+    <col min="26" max="16384" width="9.140625" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" s="8" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" s="8" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="str">
         <f>_xlfn.CONCAT("Total: ", SUM(A7,F7,K7,P7,U7))</f>
         <v>Total: 121</v>
@@ -966,659 +1033,583 @@
       <c r="O1" s="13"/>
       <c r="T1" s="4"/>
     </row>
-    <row r="2" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="19"/>
       <c r="F2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="17" t="s">
+      <c r="G2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="17" t="s">
+      <c r="I2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="19"/>
       <c r="K2" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="L2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="M2" s="17" t="s">
+      <c r="M2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="N2" s="17" t="s">
+      <c r="N2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="O2" s="19"/>
       <c r="P2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="17" t="s">
+      <c r="Q2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="R2" s="17" t="s">
+      <c r="R2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="S2" s="17" t="s">
+      <c r="S2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="T2" s="19"/>
       <c r="U2" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="V2" s="17" t="s">
+      <c r="V2" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="W2" s="17" t="s">
+      <c r="W2" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="X2" s="17" t="s">
+      <c r="X2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="Y2" s="19"/>
     </row>
-    <row r="3" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="15">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
         <f>COUNTA(B3:B60)</f>
         <v>9</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="B3" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="C3" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="19"/>
-      <c r="F3" s="15">
+      <c r="C3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F3" s="1">
         <f>COUNTA(G3:G60)</f>
         <v>10</v>
       </c>
-      <c r="G3" s="25" t="s">
-        <v>32</v>
-      </c>
-      <c r="H3" s="21" t="s">
+      <c r="G3" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="J3" s="19"/>
-      <c r="K3" s="15">
+      <c r="K3" s="1">
         <f>COUNTA(L3:L60)</f>
         <v>9</v>
       </c>
-      <c r="L3" s="16" t="s">
+      <c r="L3" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="M3" s="22" t="s">
+      <c r="M3" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="N3" s="21" t="s">
+      <c r="N3" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="O3" s="19"/>
-      <c r="P3" s="15">
+      <c r="P3" s="1">
         <f>COUNTA(Q3:Q60)</f>
         <v>11</v>
       </c>
-      <c r="Q3" s="21" t="s">
+      <c r="Q3" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="R3" s="21" t="s">
+      <c r="R3" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="S3" s="22" t="s">
+      <c r="S3" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="T3" s="19"/>
-      <c r="U3" s="15">
+      <c r="U3" s="1">
         <f>COUNTA(V3:V60)</f>
         <v>14</v>
       </c>
-      <c r="V3" s="21" t="s">
+      <c r="V3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="W3" s="22" t="s">
+      <c r="W3" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="X3" s="16" t="s">
+      <c r="X3" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="Y3" s="19"/>
     </row>
-    <row r="4" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="15">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
         <f>COUNTA(C3:C60)</f>
         <v>7</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="21" t="s">
-        <v>42</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="E4" s="19"/>
-      <c r="F4" s="15">
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="1">
         <f>COUNTA(H3:H60)</f>
         <v>7</v>
       </c>
-      <c r="G4" s="16" t="s">
-        <v>54</v>
-      </c>
-      <c r="H4" s="21" t="s">
+      <c r="G4" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="19"/>
-      <c r="K4" s="15">
+      <c r="K4" s="1">
         <f>COUNTA(M3:M60)</f>
         <v>5</v>
       </c>
-      <c r="L4" s="22" t="s">
+      <c r="L4" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="M4" s="16" t="s">
+      <c r="M4" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="N4" s="16" t="s">
+      <c r="N4" s="15" t="s">
         <v>39</v>
       </c>
-      <c r="O4" s="19"/>
-      <c r="P4" s="15">
+      <c r="P4" s="1">
         <f>COUNTA(R3:R60)</f>
         <v>5</v>
       </c>
-      <c r="Q4" s="22" t="s">
+      <c r="Q4" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="R4" s="21" t="s">
+      <c r="R4" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="S4" s="22" t="s">
+      <c r="S4" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="T4" s="19"/>
-      <c r="U4" s="15">
+      <c r="U4" s="1">
         <f>COUNTA(W3:W60)</f>
         <v>11</v>
       </c>
-      <c r="V4" s="21" t="s">
+      <c r="V4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="W4" s="21" t="s">
+      <c r="W4" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="X4" s="22" t="s">
+      <c r="X4" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="Y4" s="19"/>
     </row>
-    <row r="5" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
         <f>COUNTA(D3:D60)</f>
         <v>7</v>
       </c>
-      <c r="B5" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="D5" s="22" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="19"/>
-      <c r="F5" s="15">
+      <c r="B5" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="1">
         <f>COUNTA(I3:I60)</f>
         <v>5</v>
       </c>
-      <c r="G5" s="25" t="s">
-        <v>77</v>
-      </c>
-      <c r="H5" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="I5" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="J5" s="19"/>
-      <c r="K5" s="15">
+      <c r="G5" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="K5" s="1">
         <f>COUNTA(N3:N60)</f>
         <v>8</v>
       </c>
-      <c r="L5" s="25" t="s">
+      <c r="L5" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="M5" s="21" t="s">
+      <c r="M5" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="N5" s="21" t="s">
+      <c r="N5" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="O5" s="19"/>
-      <c r="P5" s="15">
+      <c r="P5" s="1">
         <f>COUNTA(S3:S60)</f>
         <v>6</v>
       </c>
-      <c r="Q5" s="21" t="s">
+      <c r="Q5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="R5" s="16" t="s">
+      <c r="R5" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="S5" s="25" t="s">
+      <c r="S5" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="T5" s="19"/>
-      <c r="U5" s="15">
+      <c r="U5" s="1">
         <f>COUNTA(X3:X60)</f>
         <v>7</v>
       </c>
-      <c r="V5" s="21" t="s">
+      <c r="V5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="W5" s="16" t="s">
+      <c r="W5" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="X5" s="25" t="s">
+      <c r="X5" s="20" t="s">
         <v>108</v>
       </c>
-      <c r="Y5" s="19"/>
     </row>
-    <row r="6" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="17" t="s">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="21" t="s">
-        <v>84</v>
-      </c>
-      <c r="C6" s="21" t="s">
+      <c r="B6" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="16" t="s">
+      <c r="D6" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="E6" s="19"/>
-      <c r="F6" s="23" t="s">
+      <c r="F6" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="G6" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="H6" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="I6" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="J6" s="19"/>
-      <c r="K6" s="17" t="s">
+      <c r="G6" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="K6" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="L6" s="21" t="s">
+      <c r="L6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="M6" s="21" t="s">
+      <c r="M6" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="N6" s="16" t="s">
+      <c r="N6" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="O6" s="19"/>
-      <c r="P6" s="17" t="s">
+      <c r="P6" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="Q6" s="25" t="s">
+      <c r="Q6" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="R6" s="22" t="s">
+      <c r="R6" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="S6" s="21" t="s">
+      <c r="S6" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T6" s="19"/>
-      <c r="U6" s="17" t="s">
+      <c r="U6" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="V6" s="22" t="s">
+      <c r="V6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="W6" s="16" t="s">
+      <c r="W6" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="X6" s="25" t="s">
+      <c r="X6" s="20" t="s">
         <v>110</v>
       </c>
-      <c r="Y6" s="19"/>
     </row>
-    <row r="7" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="15">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
         <f>SUM(A3:A5)</f>
         <v>23</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="B7" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="21" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>49</v>
-      </c>
-      <c r="E7" s="19"/>
-      <c r="F7" s="15">
+      <c r="C7" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>114</v>
+      </c>
+      <c r="F7" s="1">
         <f>SUM(F3:F5)</f>
         <v>22</v>
       </c>
-      <c r="G7" s="21" t="s">
-        <v>89</v>
-      </c>
-      <c r="H7" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="I7" s="22" t="s">
-        <v>98</v>
-      </c>
-      <c r="J7" s="19"/>
-      <c r="K7" s="15">
+      <c r="G7" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="K7" s="1">
         <f>SUM(K3:K5)</f>
         <v>22</v>
       </c>
-      <c r="L7" s="21" t="s">
+      <c r="L7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="M7" s="22" t="s">
+      <c r="M7" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="N7" s="25" t="s">
+      <c r="N7" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="O7" s="19"/>
-      <c r="P7" s="15">
+      <c r="P7" s="1">
         <f>SUM(P3:P5)</f>
         <v>22</v>
       </c>
-      <c r="Q7" s="16" t="s">
+      <c r="Q7" s="15" t="s">
         <v>56</v>
       </c>
-      <c r="R7" s="25" t="s">
+      <c r="R7" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="S7" s="21" t="s">
+      <c r="S7" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="T7" s="19"/>
-      <c r="U7" s="15">
+      <c r="U7" s="1">
         <f>SUM(U3:U5)</f>
         <v>32</v>
       </c>
-      <c r="V7" s="25" t="s">
+      <c r="V7" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="W7" s="22" t="s">
+      <c r="W7" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="X7" s="16" t="s">
+      <c r="X7" s="15" t="s">
         <v>12</v>
       </c>
-      <c r="Y7" s="19"/>
     </row>
-    <row r="8" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="24"/>
-      <c r="B8" s="25" t="s">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A8" s="19"/>
+      <c r="B8" s="15" t="s">
+        <v>101</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F8" s="19"/>
+      <c r="G8" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="K8" s="19"/>
+      <c r="L8" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="S8" s="15" t="s">
+        <v>105</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="W8" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="X8" s="2" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A9" s="20"/>
+      <c r="B9" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="20"/>
+      <c r="G9" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>94</v>
+      </c>
+      <c r="K9" s="20"/>
+      <c r="L9" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="U9" s="20"/>
+      <c r="V9" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="W9" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="X9" s="2" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="E8" s="19"/>
-      <c r="F8" s="24"/>
-      <c r="G8" s="21" t="s">
-        <v>91</v>
-      </c>
-      <c r="H8" s="16" t="s">
-        <v>57</v>
-      </c>
-      <c r="J8" s="19"/>
-      <c r="K8" s="24"/>
-      <c r="L8" s="16" t="s">
-        <v>68</v>
-      </c>
-      <c r="M8" s="26"/>
-      <c r="N8" s="21" t="s">
-        <v>34</v>
-      </c>
-      <c r="O8" s="19"/>
-      <c r="P8" s="24"/>
-      <c r="Q8" s="16" t="s">
-        <v>80</v>
-      </c>
-      <c r="S8" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="T8" s="19"/>
-      <c r="U8" s="15"/>
-      <c r="V8" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="W8" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="X8" s="21" t="s">
-        <v>129</v>
-      </c>
-      <c r="Y8" s="19"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="K10" s="20"/>
+      <c r="L10" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="N10" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="P10" s="20"/>
+      <c r="Q10" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="U10" s="20"/>
+      <c r="V10" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="W10" s="15" t="s">
+        <v>111</v>
+      </c>
     </row>
-    <row r="9" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="25"/>
-      <c r="B9" s="21" t="s">
-        <v>100</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="E9" s="19"/>
-      <c r="F9" s="25"/>
-      <c r="G9" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="H9" s="16" t="s">
-        <v>94</v>
-      </c>
-      <c r="J9" s="19"/>
-      <c r="K9" s="25"/>
-      <c r="L9" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="N9" s="22" t="s">
-        <v>26</v>
-      </c>
-      <c r="O9" s="19"/>
-      <c r="P9" s="25"/>
-      <c r="Q9" s="16" t="s">
-        <v>63</v>
-      </c>
-      <c r="T9" s="19"/>
-      <c r="U9" s="25"/>
-      <c r="V9" s="25" t="s">
-        <v>109</v>
-      </c>
-      <c r="W9" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="X9" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="Y9" s="19"/>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="B11" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="G11" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="L11" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q11" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="W11" s="15" t="s">
+        <v>119</v>
+      </c>
     </row>
-    <row r="10" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="25"/>
-      <c r="B10" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="E10" s="19"/>
-      <c r="F10" s="25"/>
-      <c r="G10" s="21" t="s">
-        <v>95</v>
-      </c>
-      <c r="J10" s="19"/>
-      <c r="K10" s="25"/>
-      <c r="L10" s="21" t="s">
-        <v>99</v>
-      </c>
-      <c r="N10" s="16" t="s">
-        <v>103</v>
-      </c>
-      <c r="O10" s="19"/>
-      <c r="P10" s="25"/>
-      <c r="Q10" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="T10" s="19"/>
-      <c r="U10" s="25"/>
-      <c r="V10" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="W10" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="Y10" s="19"/>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="G12" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="Q12" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="W12" s="15" t="s">
+        <v>120</v>
+      </c>
     </row>
-    <row r="11" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="15"/>
-      <c r="B11" s="25" t="s">
-        <v>112</v>
-      </c>
-      <c r="E11" s="19"/>
-      <c r="F11" s="15"/>
-      <c r="G11" s="21" t="s">
-        <v>96</v>
-      </c>
-      <c r="J11" s="19"/>
-      <c r="K11" s="15"/>
-      <c r="L11" s="21" t="s">
-        <v>117</v>
-      </c>
-      <c r="O11" s="19"/>
-      <c r="P11" s="15"/>
-      <c r="Q11" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="T11" s="19"/>
-      <c r="U11" s="15"/>
-      <c r="V11" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="W11" s="16" t="s">
-        <v>119</v>
-      </c>
-      <c r="Y11" s="19"/>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="Q13" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="W13" s="15" t="s">
+        <v>128</v>
+      </c>
     </row>
-    <row r="12" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="15"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="15"/>
-      <c r="G12" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="J12" s="19"/>
-      <c r="K12" s="15"/>
-      <c r="O12" s="19"/>
-      <c r="P12" s="15"/>
-      <c r="Q12" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="T12" s="19"/>
-      <c r="U12" s="15"/>
-      <c r="V12" s="21" t="s">
-        <v>123</v>
-      </c>
-      <c r="W12" s="16" t="s">
-        <v>120</v>
-      </c>
-      <c r="Y12" s="19"/>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="V14" s="2" t="s">
+        <v>125</v>
+      </c>
     </row>
-    <row r="13" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="15"/>
-      <c r="J13" s="19"/>
-      <c r="K13" s="15"/>
-      <c r="O13" s="19"/>
-      <c r="P13" s="15"/>
-      <c r="Q13" s="21" t="s">
-        <v>104</v>
-      </c>
-      <c r="T13" s="19"/>
-      <c r="U13" s="15"/>
-      <c r="V13" s="21" t="s">
-        <v>124</v>
-      </c>
-      <c r="W13" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="Y13" s="19"/>
-    </row>
-    <row r="14" spans="1:25" s="20" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="15"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="15"/>
-      <c r="J14" s="19"/>
-      <c r="K14" s="15"/>
-      <c r="O14" s="19"/>
-      <c r="P14" s="15"/>
-      <c r="T14" s="19"/>
-      <c r="U14" s="15"/>
-      <c r="V14" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="Y14" s="19"/>
-    </row>
-    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="V15" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.25">
       <c r="V16" s="3" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="17" spans="17:17" x14ac:dyDescent="0.3">
+    <row r="17" spans="17:17" x14ac:dyDescent="0.25">
       <c r="Q17" s="14"/>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="G3:I21">
+    <sortCondition sortBy="cellColor" ref="G3:G21" dxfId="8"/>
+    <sortCondition sortBy="cellColor" ref="H3:H21" dxfId="7"/>
+    <sortCondition sortBy="cellColor" ref="I3:I21" dxfId="6"/>
+    <sortCondition sortBy="cellColor" ref="G3:G21" dxfId="5"/>
+    <sortCondition sortBy="cellColor" ref="H3:H21" dxfId="4"/>
+    <sortCondition sortBy="cellColor" ref="I3:I21" dxfId="3"/>
+    <sortCondition sortBy="cellColor" ref="G3:G21" dxfId="2"/>
+    <sortCondition sortBy="cellColor" ref="I3:I21" dxfId="1"/>
+    <sortCondition sortBy="cellColor" ref="G3:G21" dxfId="0"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
added the rest of the cards
</commit_message>
<xml_diff>
--- a/Set1Layout.xlsx
+++ b/Set1Layout.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Spark\Documents\CardGame\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2154F625-4C11-4059-8CDF-EA7FD261F6B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C187B856-34DC-4157-9CCB-30EB8B771F13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15345" xr2:uid="{F1BE6F00-F159-4957-8E4B-273D781E3C31}"/>
   </bookViews>
@@ -1212,7 +1212,7 @@
       <c r="R4" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="S4" s="3" t="s">
+      <c r="S4" s="20" t="s">
         <v>59</v>
       </c>
       <c r="U4" s="1">
@@ -1336,7 +1336,7 @@
       <c r="P6" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="Q6" s="20" t="s">
+      <c r="Q6" s="3" t="s">
         <v>23</v>
       </c>
       <c r="R6" s="3" t="s">

</xml_diff>